<commit_message>
final: nettoyage et README
</commit_message>
<xml_diff>
--- a/documents/conceptualisation/Spécifications/Specifications.xlsx
+++ b/documents/conceptualisation/Spécifications/Specifications.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell Pro\Desktop\EXAMEN_2026\BACKEND_ADELINE-SIVAZ_2026\R&amp;D - supports de travail\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell Pro\Desktop\EXAMEN_2026\BACKEND_ADELINE-SIVAZ_2026\qdm-adeline\documents\conceptualisation\Spécifications\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63C488F6-FE3D-4BEA-93A9-9C95C350EC18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{481C51E6-1F2F-42D2-876D-3534556D4808}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="controleur" sheetId="1" r:id="rId1"/>

</xml_diff>